<commit_message>
Admin: README section on add/change/hide/remove products; notes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sienna-art-studio-admin/samples/sienna-products-import.xlsx
+++ b/sienna-art-studio-admin/samples/sienna-products-import.xlsx
@@ -159,7 +159,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1238" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="392">
   <si>
     <t>How to use this file</t>
   </si>
@@ -459,6 +459,63 @@
   </si>
   <si>
     <t>The product is saved but hidden.</t>
+  </si>
+  <si>
+    <t>Adding, changing, hiding and removing products</t>
+  </si>
+  <si>
+    <t>Add a new product</t>
+  </si>
+  <si>
+    <t>Add its row(s) at the bottom of the Products tab with a NEW Product Code and a NEW SKU, then upload. It is CREATED. If Status = active it shows on the site right away.</t>
+  </si>
+  <si>
+    <t>Change a product</t>
+  </si>
+  <si>
+    <t>Keep its Product Code and SKU, change the cells, upload. It is UPDATED. A cell with - is left exactly as it is on the site.</t>
+  </si>
+  <si>
+    <t>Hide a product (recommended)</t>
+  </si>
+  <si>
+    <t>Set Status to draft and upload. The product stays in the store but disappears from the site. Set it back to active to show it again.</t>
+  </si>
+  <si>
+    <t>Delete a product for good</t>
+  </si>
+  <si>
+    <t>The panel NEVER deletes products, on purpose (a wrong file must not wipe the shop). Delete it in Shopify: Admin &gt; Products &gt; open the product &gt; the three dots &gt; Delete product.</t>
+  </si>
+  <si>
+    <t>Remove a row from this Excel</t>
+  </si>
+  <si>
+    <t>Does nothing to the store. The product stays on the site. Use Status = draft to hide it, or delete it in Shopify.</t>
+  </si>
+  <si>
+    <t>Remove a category</t>
+  </si>
+  <si>
+    <t>Delete its row in the Categories tab and upload: it disappears from the site menu. The collection itself stays in Shopify (delete it there if you want).</t>
+  </si>
+  <si>
+    <t>Always run the Dry run first</t>
+  </si>
+  <si>
+    <t>Tick "Dry run" in the panel: it shows create / update for every row and writes nothing. Existing products must say update, only new ones create. If an old product says create, STOP and ask the developer.</t>
+  </si>
+  <si>
+    <t>Product made in Shopify by hand</t>
+  </si>
+  <si>
+    <t>The panel finds a product by its SKU. If the product in Shopify has an empty SKU, the panel cannot find it and makes a COPY. Type the SKU into the product in Shopify first, then upload.</t>
+  </si>
+  <si>
+    <t>Test with one product</t>
+  </si>
+  <si>
+    <t>In the panel, type the Product Code in "Only these product codes" to touch only that product. Leave it empty to import everything. Categories and the site menu are always updated.</t>
   </si>
   <si>
     <t>Name</t>
@@ -1747,7 +1804,7 @@
   <sheetPr>
     <tabColor rgb="FFC0504D"/>
   </sheetPr>
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B77"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2260,8 +2317,86 @@
         <v>99</v>
       </c>
     </row>
+    <row r="68" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B68" s="5"/>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A4:B4"/>
@@ -2273,9 +2408,10 @@
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="A55:B55"/>
     <mergeCell ref="A63:B63"/>
+    <mergeCell ref="A68:B68"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2284,7 +2420,7 @@
   <sheetPr>
     <tabColor rgb="FF4F81BD"/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -2299,10 +2435,10 @@
         <v>81</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>85</v>
@@ -2316,39 +2452,39 @@
     </row>
     <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>94</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>94</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>94</v>
@@ -2356,13 +2492,13 @@
     </row>
     <row r="4" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>94</v>
@@ -2376,19 +2512,19 @@
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>94</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>94</v>
@@ -2396,19 +2532,19 @@
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>94</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>94</v>
@@ -2416,19 +2552,19 @@
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>94</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>94</v>
@@ -2436,39 +2572,39 @@
     </row>
     <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>94</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>94</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>94</v>
@@ -2476,19 +2612,19 @@
     </row>
     <row r="10" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>94</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>94</v>
@@ -2496,39 +2632,39 @@
     </row>
     <row r="11" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>94</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>94</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>94</v>
@@ -2536,13 +2672,13 @@
     </row>
     <row r="13" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>94</v>
@@ -2556,13 +2692,13 @@
     </row>
     <row r="14" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>94</v>
@@ -2576,33 +2712,33 @@
     </row>
     <row r="15" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>94</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>94</v>
@@ -2616,13 +2752,13 @@
     </row>
     <row r="17" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>94</v>
@@ -2636,13 +2772,13 @@
     </row>
     <row r="18" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>94</v>
@@ -2656,13 +2792,13 @@
     </row>
     <row r="19" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>94</v>
@@ -2674,47 +2810,6 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <dataValidations count="4">
@@ -2732,7 +2827,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -2742,7 +2837,7 @@
   <sheetPr>
     <tabColor rgb="FF9BBB59"/>
   </sheetPr>
-  <dimension ref="A1:Y300"/>
+  <dimension ref="A1:Y56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2771,25 +2866,25 @@
         <v>27</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>35</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>70</v>
@@ -2798,22 +2893,22 @@
         <v>72</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="O1" s="6" t="s">
         <v>29</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>37</v>
@@ -2822,42 +2917,42 @@
         <v>33</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="T1" s="7" t="s">
         <v>63</v>
       </c>
       <c r="U1" s="7" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="V1" s="7" t="s">
-        <v>150</v>
+        <v>169</v>
       </c>
       <c r="W1" s="7" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
       <c r="X1" s="7" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="Y1" s="7" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>94</v>
@@ -2866,13 +2961,13 @@
         <v>94</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="K2" s="9" t="s">
         <v>94</v>
@@ -2887,7 +2982,7 @@
         <v>94</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="P2" s="9">
         <v>109.95</v>
@@ -2905,7 +3000,7 @@
         <v>94</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>160</v>
+        <v>179</v>
       </c>
       <c r="V2" s="9" t="s">
         <v>94</v>
@@ -2922,16 +3017,16 @@
     </row>
     <row r="3" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>161</v>
+        <v>180</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>94</v>
@@ -2940,13 +3035,13 @@
         <v>94</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J3" s="9" t="s">
         <v>94</v>
@@ -2964,7 +3059,7 @@
         <v>94</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>161</v>
+        <v>180</v>
       </c>
       <c r="P3" s="9">
         <v>109.99</v>
@@ -2982,13 +3077,13 @@
         <v>94</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="V3" s="9" t="s">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="W3" s="9" t="s">
-        <v>166</v>
+        <v>185</v>
       </c>
       <c r="X3" s="9" t="s">
         <v>94</v>
@@ -2999,16 +3094,16 @@
     </row>
     <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>168</v>
+        <v>187</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>94</v>
@@ -3017,13 +3112,13 @@
         <v>94</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>94</v>
@@ -3041,7 +3136,7 @@
         <v>94</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="P4" s="9">
         <v>109.99</v>
@@ -3059,13 +3154,13 @@
         <v>94</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="V4" s="9" t="s">
-        <v>170</v>
+        <v>189</v>
       </c>
       <c r="W4" s="9" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="X4" s="9" t="s">
         <v>94</v>
@@ -3076,16 +3171,16 @@
     </row>
     <row r="5" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>94</v>
@@ -3094,13 +3189,13 @@
         <v>94</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J5" s="9" t="s">
         <v>94</v>
@@ -3118,7 +3213,7 @@
         <v>94</v>
       </c>
       <c r="O5" s="9" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
       <c r="P5" s="9">
         <v>14.99</v>
@@ -3136,10 +3231,10 @@
         <v>94</v>
       </c>
       <c r="U5" s="9" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="V5" s="9" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="W5" s="9" t="s">
         <v>94</v>
@@ -3153,31 +3248,31 @@
     </row>
     <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>157</v>
-      </c>
       <c r="I6" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J6" s="9" t="s">
         <v>94</v>
@@ -3195,7 +3290,7 @@
         <v>94</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="P6" s="9">
         <v>14.99</v>
@@ -3213,10 +3308,10 @@
         <v>94</v>
       </c>
       <c r="U6" s="9" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="V6" s="9" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="W6" s="9" t="s">
         <v>94</v>
@@ -3230,16 +3325,16 @@
     </row>
     <row r="7" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>94</v>
@@ -3248,13 +3343,13 @@
         <v>94</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>94</v>
@@ -3272,7 +3367,7 @@
         <v>94</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="P7" s="9">
         <v>49.95</v>
@@ -3290,7 +3385,7 @@
         <v>94</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="V7" s="9" t="s">
         <v>94</v>
@@ -3307,32 +3402,32 @@
     </row>
     <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="I8" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>164</v>
-      </c>
       <c r="J8" s="9" t="s">
         <v>94</v>
       </c>
@@ -3349,7 +3444,7 @@
         <v>94</v>
       </c>
       <c r="O8" s="9" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="P8" s="9">
         <v>49.95</v>
@@ -3367,7 +3462,7 @@
         <v>94</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="V8" s="9" t="s">
         <v>94</v>
@@ -3384,16 +3479,16 @@
     </row>
     <row r="9" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>187</v>
+        <v>206</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>94</v>
@@ -3402,13 +3497,13 @@
         <v>94</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>94</v>
@@ -3426,7 +3521,7 @@
         <v>94</v>
       </c>
       <c r="O9" s="9" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
       <c r="P9" s="9">
         <v>49.95</v>
@@ -3444,7 +3539,7 @@
         <v>94</v>
       </c>
       <c r="U9" s="9" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
       <c r="V9" s="9" t="s">
         <v>94</v>
@@ -3461,16 +3556,16 @@
     </row>
     <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>94</v>
@@ -3479,13 +3574,13 @@
         <v>94</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>94</v>
@@ -3503,7 +3598,7 @@
         <v>94</v>
       </c>
       <c r="O10" s="9" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="P10" s="9">
         <v>14.99</v>
@@ -3521,10 +3616,10 @@
         <v>94</v>
       </c>
       <c r="U10" s="9" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="V10" s="9" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="W10" s="9" t="s">
         <v>94</v>
@@ -3538,31 +3633,31 @@
     </row>
     <row r="11" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="G11" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>174</v>
-      </c>
       <c r="H11" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>94</v>
@@ -3580,7 +3675,7 @@
         <v>94</v>
       </c>
       <c r="O11" s="9" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="P11" s="9">
         <v>9.99</v>
@@ -3598,10 +3693,10 @@
         <v>94</v>
       </c>
       <c r="U11" s="9" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
       <c r="V11" s="9" t="s">
-        <v>196</v>
+        <v>215</v>
       </c>
       <c r="W11" s="9" t="s">
         <v>94</v>
@@ -3615,16 +3710,16 @@
     </row>
     <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>94</v>
@@ -3633,13 +3728,13 @@
         <v>94</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>94</v>
@@ -3657,7 +3752,7 @@
         <v>94</v>
       </c>
       <c r="O12" s="9" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="P12" s="9">
         <v>9.99</v>
@@ -3675,10 +3770,10 @@
         <v>94</v>
       </c>
       <c r="U12" s="9" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="V12" s="9" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="W12" s="9" t="s">
         <v>94</v>
@@ -3692,16 +3787,16 @@
     </row>
     <row r="13" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>94</v>
@@ -3710,13 +3805,13 @@
         <v>94</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J13" s="9" t="s">
         <v>94</v>
@@ -3734,7 +3829,7 @@
         <v>94</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="P13" s="9">
         <v>14.99</v>
@@ -3752,10 +3847,10 @@
         <v>94</v>
       </c>
       <c r="U13" s="9" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="V13" s="9" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="W13" s="9" t="s">
         <v>94</v>
@@ -3769,16 +3864,16 @@
     </row>
     <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>206</v>
+        <v>225</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>94</v>
@@ -3787,13 +3882,13 @@
         <v>94</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J14" s="9" t="s">
         <v>94</v>
@@ -3811,7 +3906,7 @@
         <v>94</v>
       </c>
       <c r="O14" s="9" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
       <c r="P14" s="9">
         <v>9.99</v>
@@ -3829,10 +3924,10 @@
         <v>94</v>
       </c>
       <c r="U14" s="9" t="s">
-        <v>207</v>
+        <v>226</v>
       </c>
       <c r="V14" s="9" t="s">
-        <v>208</v>
+        <v>227</v>
       </c>
       <c r="W14" s="9" t="s">
         <v>94</v>
@@ -3846,16 +3941,16 @@
     </row>
     <row r="15" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>209</v>
+        <v>228</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>210</v>
+        <v>229</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>94</v>
@@ -3864,13 +3959,13 @@
         <v>94</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>94</v>
@@ -3888,7 +3983,7 @@
         <v>94</v>
       </c>
       <c r="O15" s="9" t="s">
-        <v>209</v>
+        <v>228</v>
       </c>
       <c r="P15" s="9">
         <v>9.99</v>
@@ -3906,10 +4001,10 @@
         <v>94</v>
       </c>
       <c r="U15" s="9" t="s">
-        <v>211</v>
+        <v>230</v>
       </c>
       <c r="V15" s="9" t="s">
-        <v>212</v>
+        <v>231</v>
       </c>
       <c r="W15" s="9" t="s">
         <v>94</v>
@@ -3923,16 +4018,16 @@
     </row>
     <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>94</v>
@@ -3941,13 +4036,13 @@
         <v>94</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J16" s="9" t="s">
         <v>94</v>
@@ -3965,7 +4060,7 @@
         <v>94</v>
       </c>
       <c r="O16" s="9" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
       <c r="P16" s="9">
         <v>12.99</v>
@@ -3983,10 +4078,10 @@
         <v>94</v>
       </c>
       <c r="U16" s="9" t="s">
-        <v>215</v>
+        <v>234</v>
       </c>
       <c r="V16" s="9" t="s">
-        <v>216</v>
+        <v>235</v>
       </c>
       <c r="W16" s="9" t="s">
         <v>94</v>
@@ -4000,16 +4095,16 @@
     </row>
     <row r="17" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>218</v>
+        <v>237</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>94</v>
@@ -4018,13 +4113,13 @@
         <v>94</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J17" s="9" t="s">
         <v>94</v>
@@ -4042,7 +4137,7 @@
         <v>94</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="P17" s="9">
         <v>14.99</v>
@@ -4060,10 +4155,10 @@
         <v>94</v>
       </c>
       <c r="U17" s="9" t="s">
-        <v>219</v>
+        <v>238</v>
       </c>
       <c r="V17" s="9" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="W17" s="9" t="s">
         <v>94</v>
@@ -4077,16 +4172,16 @@
     </row>
     <row r="18" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>94</v>
@@ -4095,13 +4190,13 @@
         <v>94</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J18" s="9" t="s">
         <v>94</v>
@@ -4119,7 +4214,7 @@
         <v>94</v>
       </c>
       <c r="O18" s="9" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="P18" s="9">
         <v>14.99</v>
@@ -4137,10 +4232,10 @@
         <v>94</v>
       </c>
       <c r="U18" s="9" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
       <c r="V18" s="9" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
       <c r="W18" s="9" t="s">
         <v>94</v>
@@ -4154,16 +4249,16 @@
     </row>
     <row r="19" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>225</v>
+        <v>244</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>226</v>
+        <v>245</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>94</v>
@@ -4172,13 +4267,13 @@
         <v>94</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J19" s="9" t="s">
         <v>94</v>
@@ -4196,7 +4291,7 @@
         <v>94</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>225</v>
+        <v>244</v>
       </c>
       <c r="P19" s="9">
         <v>12.99</v>
@@ -4214,10 +4309,10 @@
         <v>94</v>
       </c>
       <c r="U19" s="9" t="s">
-        <v>227</v>
+        <v>246</v>
       </c>
       <c r="V19" s="9" t="s">
-        <v>228</v>
+        <v>247</v>
       </c>
       <c r="W19" s="9" t="s">
         <v>94</v>
@@ -4231,16 +4326,16 @@
     </row>
     <row r="20" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>229</v>
+        <v>248</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>94</v>
@@ -4249,13 +4344,13 @@
         <v>94</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J20" s="9" t="s">
         <v>94</v>
@@ -4273,7 +4368,7 @@
         <v>94</v>
       </c>
       <c r="O20" s="9" t="s">
-        <v>229</v>
+        <v>248</v>
       </c>
       <c r="P20" s="9">
         <v>14.99</v>
@@ -4291,10 +4386,10 @@
         <v>94</v>
       </c>
       <c r="U20" s="9" t="s">
-        <v>231</v>
+        <v>250</v>
       </c>
       <c r="V20" s="9" t="s">
-        <v>232</v>
+        <v>251</v>
       </c>
       <c r="W20" s="9" t="s">
         <v>94</v>
@@ -4308,16 +4403,16 @@
     </row>
     <row r="21" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>233</v>
+        <v>252</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>234</v>
+        <v>253</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>94</v>
@@ -4326,13 +4421,13 @@
         <v>94</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J21" s="9" t="s">
         <v>94</v>
@@ -4350,7 +4445,7 @@
         <v>94</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>233</v>
+        <v>252</v>
       </c>
       <c r="P21" s="9">
         <v>14.99</v>
@@ -4368,10 +4463,10 @@
         <v>94</v>
       </c>
       <c r="U21" s="9" t="s">
-        <v>235</v>
+        <v>254</v>
       </c>
       <c r="V21" s="9" t="s">
-        <v>236</v>
+        <v>255</v>
       </c>
       <c r="W21" s="9" t="s">
         <v>94</v>
@@ -4385,16 +4480,16 @@
     </row>
     <row r="22" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>94</v>
@@ -4403,13 +4498,13 @@
         <v>94</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J22" s="9" t="s">
         <v>94</v>
@@ -4427,7 +4522,7 @@
         <v>94</v>
       </c>
       <c r="O22" s="9" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
       <c r="P22" s="9">
         <v>12.99</v>
@@ -4445,10 +4540,10 @@
         <v>94</v>
       </c>
       <c r="U22" s="9" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
       <c r="V22" s="9" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
       <c r="W22" s="9" t="s">
         <v>94</v>
@@ -4462,16 +4557,16 @@
     </row>
     <row r="23" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>94</v>
@@ -4480,13 +4575,13 @@
         <v>94</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J23" s="9" t="s">
         <v>94</v>
@@ -4504,7 +4599,7 @@
         <v>94</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
       <c r="P23" s="9">
         <v>14.99</v>
@@ -4522,10 +4617,10 @@
         <v>94</v>
       </c>
       <c r="U23" s="9" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
       <c r="V23" s="9" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
       <c r="W23" s="9" t="s">
         <v>94</v>
@@ -4539,16 +4634,16 @@
     </row>
     <row r="24" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E24" s="9" t="s">
         <v>94</v>
@@ -4557,13 +4652,13 @@
         <v>94</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J24" s="9" t="s">
         <v>94</v>
@@ -4581,7 +4676,7 @@
         <v>94</v>
       </c>
       <c r="O24" s="9" t="s">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="P24" s="9">
         <v>14.99</v>
@@ -4599,10 +4694,10 @@
         <v>94</v>
       </c>
       <c r="U24" s="9" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
       <c r="V24" s="9" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="W24" s="9" t="s">
         <v>94</v>
@@ -4616,16 +4711,16 @@
     </row>
     <row r="25" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>249</v>
+        <v>268</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>250</v>
+        <v>269</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>94</v>
@@ -4634,13 +4729,13 @@
         <v>94</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J25" s="9" t="s">
         <v>94</v>
@@ -4658,7 +4753,7 @@
         <v>94</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>249</v>
+        <v>268</v>
       </c>
       <c r="P25" s="9">
         <v>12.99</v>
@@ -4676,10 +4771,10 @@
         <v>94</v>
       </c>
       <c r="U25" s="9" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
       <c r="V25" s="9" t="s">
-        <v>252</v>
+        <v>271</v>
       </c>
       <c r="W25" s="9" t="s">
         <v>94</v>
@@ -4693,16 +4788,16 @@
     </row>
     <row r="26" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>254</v>
+        <v>273</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>94</v>
@@ -4711,13 +4806,13 @@
         <v>94</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J26" s="9" t="s">
         <v>94</v>
@@ -4735,7 +4830,7 @@
         <v>94</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="P26" s="9">
         <v>12.99</v>
@@ -4753,10 +4848,10 @@
         <v>94</v>
       </c>
       <c r="U26" s="9" t="s">
-        <v>255</v>
+        <v>274</v>
       </c>
       <c r="V26" s="9" t="s">
-        <v>256</v>
+        <v>275</v>
       </c>
       <c r="W26" s="9" t="s">
         <v>94</v>
@@ -4770,16 +4865,16 @@
     </row>
     <row r="27" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>257</v>
+        <v>276</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>258</v>
+        <v>277</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>94</v>
@@ -4788,13 +4883,13 @@
         <v>94</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J27" s="9" t="s">
         <v>94</v>
@@ -4812,7 +4907,7 @@
         <v>94</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>257</v>
+        <v>276</v>
       </c>
       <c r="P27" s="9">
         <v>14.99</v>
@@ -4830,10 +4925,10 @@
         <v>94</v>
       </c>
       <c r="U27" s="9" t="s">
-        <v>259</v>
+        <v>278</v>
       </c>
       <c r="V27" s="9" t="s">
-        <v>260</v>
+        <v>279</v>
       </c>
       <c r="W27" s="9" t="s">
         <v>94</v>
@@ -4847,16 +4942,16 @@
     </row>
     <row r="28" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>262</v>
+        <v>281</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E28" s="9" t="s">
         <v>94</v>
@@ -4865,13 +4960,13 @@
         <v>94</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J28" s="9" t="s">
         <v>94</v>
@@ -4889,7 +4984,7 @@
         <v>94</v>
       </c>
       <c r="O28" s="9" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
       <c r="P28" s="9">
         <v>14.99</v>
@@ -4907,10 +5002,10 @@
         <v>94</v>
       </c>
       <c r="U28" s="9" t="s">
-        <v>263</v>
+        <v>282</v>
       </c>
       <c r="V28" s="9" t="s">
-        <v>264</v>
+        <v>283</v>
       </c>
       <c r="W28" s="9" t="s">
         <v>94</v>
@@ -4924,16 +5019,16 @@
     </row>
     <row r="29" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>265</v>
+        <v>284</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>266</v>
+        <v>285</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>94</v>
@@ -4942,13 +5037,13 @@
         <v>94</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J29" s="9" t="s">
         <v>94</v>
@@ -4966,7 +5061,7 @@
         <v>94</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>265</v>
+        <v>284</v>
       </c>
       <c r="P29" s="9">
         <v>15.99</v>
@@ -4984,10 +5079,10 @@
         <v>94</v>
       </c>
       <c r="U29" s="9" t="s">
-        <v>267</v>
+        <v>286</v>
       </c>
       <c r="V29" s="9" t="s">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="W29" s="9" t="s">
         <v>94</v>
@@ -5001,16 +5096,16 @@
     </row>
     <row r="30" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E30" s="9" t="s">
         <v>94</v>
@@ -5019,13 +5114,13 @@
         <v>94</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J30" s="9" t="s">
         <v>94</v>
@@ -5043,7 +5138,7 @@
         <v>94</v>
       </c>
       <c r="O30" s="9" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="P30" s="9">
         <v>9.99</v>
@@ -5061,10 +5156,10 @@
         <v>94</v>
       </c>
       <c r="U30" s="9" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
       <c r="V30" s="9" t="s">
-        <v>272</v>
+        <v>291</v>
       </c>
       <c r="W30" s="9" t="s">
         <v>94</v>
@@ -5078,16 +5173,16 @@
     </row>
     <row r="31" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>273</v>
+        <v>292</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>94</v>
@@ -5096,22 +5191,22 @@
         <v>94</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J31" s="9" t="s">
         <v>94</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="L31" s="9" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="M31" s="9" t="s">
         <v>94</v>
@@ -5120,7 +5215,7 @@
         <v>94</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>273</v>
+        <v>292</v>
       </c>
       <c r="P31" s="9">
         <v>14.99</v>
@@ -5135,7 +5230,7 @@
         <v>227</v>
       </c>
       <c r="T31" s="9" t="s">
-        <v>277</v>
+        <v>296</v>
       </c>
       <c r="U31" s="9" t="s">
         <v>94</v>
@@ -5155,7 +5250,7 @@
     </row>
     <row r="32" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>273</v>
+        <v>292</v>
       </c>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
@@ -5167,10 +5262,10 @@
       <c r="I32" s="10"/>
       <c r="J32" s="10"/>
       <c r="K32" s="2" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>278</v>
+        <v>297</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>94</v>
@@ -5179,7 +5274,7 @@
         <v>94</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>279</v>
+        <v>298</v>
       </c>
       <c r="P32" s="2">
         <v>14.99</v>
@@ -5194,7 +5289,7 @@
         <v>227</v>
       </c>
       <c r="T32" s="2" t="s">
-        <v>280</v>
+        <v>299</v>
       </c>
       <c r="U32" s="10"/>
       <c r="V32" s="10"/>
@@ -5204,16 +5299,16 @@
     </row>
     <row r="33" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>281</v>
+        <v>300</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>282</v>
+        <v>301</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>94</v>
@@ -5222,13 +5317,13 @@
         <v>94</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J33" s="9" t="s">
         <v>94</v>
@@ -5246,7 +5341,7 @@
         <v>94</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>281</v>
+        <v>300</v>
       </c>
       <c r="P33" s="9">
         <v>19.99</v>
@@ -5264,10 +5359,10 @@
         <v>94</v>
       </c>
       <c r="U33" s="9" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
       <c r="V33" s="9" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="W33" s="9" t="s">
         <v>94</v>
@@ -5281,16 +5376,16 @@
     </row>
     <row r="34" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>285</v>
+        <v>304</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>286</v>
+        <v>305</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E34" s="9" t="s">
         <v>94</v>
@@ -5299,13 +5394,13 @@
         <v>94</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J34" s="9" t="s">
         <v>94</v>
@@ -5323,7 +5418,7 @@
         <v>94</v>
       </c>
       <c r="O34" s="9" t="s">
-        <v>285</v>
+        <v>304</v>
       </c>
       <c r="P34" s="9">
         <v>12.99</v>
@@ -5341,10 +5436,10 @@
         <v>94</v>
       </c>
       <c r="U34" s="9" t="s">
-        <v>287</v>
+        <v>306</v>
       </c>
       <c r="V34" s="9" t="s">
-        <v>288</v>
+        <v>307</v>
       </c>
       <c r="W34" s="9" t="s">
         <v>94</v>
@@ -5358,16 +5453,16 @@
     </row>
     <row r="35" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>290</v>
+        <v>309</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>94</v>
@@ -5376,13 +5471,13 @@
         <v>94</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J35" s="9" t="s">
         <v>94</v>
@@ -5400,7 +5495,7 @@
         <v>94</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
       <c r="P35" s="9">
         <v>14.99</v>
@@ -5418,10 +5513,10 @@
         <v>94</v>
       </c>
       <c r="U35" s="9" t="s">
-        <v>291</v>
+        <v>310</v>
       </c>
       <c r="V35" s="9" t="s">
-        <v>292</v>
+        <v>311</v>
       </c>
       <c r="W35" s="9" t="s">
         <v>94</v>
@@ -5435,16 +5530,16 @@
     </row>
     <row r="36" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>293</v>
+        <v>312</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>294</v>
+        <v>313</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>94</v>
@@ -5453,13 +5548,13 @@
         <v>94</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J36" s="9" t="s">
         <v>94</v>
@@ -5477,7 +5572,7 @@
         <v>94</v>
       </c>
       <c r="O36" s="9" t="s">
-        <v>293</v>
+        <v>312</v>
       </c>
       <c r="P36" s="9">
         <v>9.99</v>
@@ -5495,10 +5590,10 @@
         <v>94</v>
       </c>
       <c r="U36" s="9" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
       <c r="V36" s="9" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="W36" s="9" t="s">
         <v>94</v>
@@ -5512,49 +5607,49 @@
     </row>
     <row r="37" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>298</v>
+        <v>317</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>299</v>
+        <v>318</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>94</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I37" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J37" s="9" t="s">
         <v>94</v>
       </c>
       <c r="K37" s="9" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="L37" s="9" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
       <c r="M37" s="9" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="O37" s="9" t="s">
-        <v>304</v>
+        <v>323</v>
       </c>
       <c r="P37" s="9">
         <v>145.95</v>
@@ -5569,7 +5664,7 @@
         <v>94</v>
       </c>
       <c r="T37" s="9" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="U37" s="9" t="s">
         <v>94</v>
@@ -5589,7 +5684,7 @@
     </row>
     <row r="38" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
       <c r="B38" s="10"/>
       <c r="C38" s="10"/>
@@ -5601,19 +5696,19 @@
       <c r="I38" s="10"/>
       <c r="J38" s="10"/>
       <c r="K38" s="2" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
       <c r="O38" s="2" t="s">
-        <v>306</v>
+        <v>325</v>
       </c>
       <c r="P38" s="2">
         <v>179.95</v>
@@ -5628,7 +5723,7 @@
         <v>94</v>
       </c>
       <c r="T38" s="2" t="s">
-        <v>307</v>
+        <v>326</v>
       </c>
       <c r="U38" s="10"/>
       <c r="V38" s="10"/>
@@ -5638,7 +5733,7 @@
     </row>
     <row r="39" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
       <c r="B39" s="10"/>
       <c r="C39" s="10"/>
@@ -5650,19 +5745,19 @@
       <c r="I39" s="10"/>
       <c r="J39" s="10"/>
       <c r="K39" s="2" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="O39" s="2" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="P39" s="2">
         <v>145.95</v>
@@ -5677,7 +5772,7 @@
         <v>94</v>
       </c>
       <c r="T39" s="2" t="s">
-        <v>310</v>
+        <v>329</v>
       </c>
       <c r="U39" s="10"/>
       <c r="V39" s="10"/>
@@ -5687,7 +5782,7 @@
     </row>
     <row r="40" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
@@ -5699,19 +5794,19 @@
       <c r="I40" s="10"/>
       <c r="J40" s="10"/>
       <c r="K40" s="2" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
       <c r="O40" s="2" t="s">
-        <v>311</v>
+        <v>330</v>
       </c>
       <c r="P40" s="2">
         <v>179.95</v>
@@ -5726,7 +5821,7 @@
         <v>94</v>
       </c>
       <c r="T40" s="2" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="U40" s="10"/>
       <c r="V40" s="10"/>
@@ -5736,31 +5831,31 @@
     </row>
     <row r="41" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>314</v>
+        <v>333</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>315</v>
+        <v>334</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J41" s="9" t="s">
         <v>94</v>
@@ -5778,7 +5873,7 @@
         <v>94</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
       <c r="P41" s="9">
         <v>145.95</v>
@@ -5796,7 +5891,7 @@
         <v>94</v>
       </c>
       <c r="U41" s="9" t="s">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="V41" s="9" t="s">
         <v>94</v>
@@ -5813,40 +5908,40 @@
     </row>
     <row r="42" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>319</v>
+        <v>338</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>321</v>
+        <v>340</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>94</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I42" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J42" s="9" t="s">
         <v>94</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="L42" s="9" t="s">
-        <v>323</v>
+        <v>342</v>
       </c>
       <c r="M42" s="9" t="s">
         <v>94</v>
@@ -5855,7 +5950,7 @@
         <v>94</v>
       </c>
       <c r="O42" s="9" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="P42" s="9">
         <v>18.95</v>
@@ -5870,7 +5965,7 @@
         <v>286</v>
       </c>
       <c r="T42" s="9" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="U42" s="9" t="s">
         <v>94</v>
@@ -5890,7 +5985,7 @@
     </row>
     <row r="43" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>319</v>
+        <v>338</v>
       </c>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
@@ -5902,10 +5997,10 @@
       <c r="I43" s="10"/>
       <c r="J43" s="10"/>
       <c r="K43" s="2" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
       <c r="M43" s="2" t="s">
         <v>94</v>
@@ -5914,7 +6009,7 @@
         <v>94</v>
       </c>
       <c r="O43" s="2" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="P43" s="2">
         <v>18.95</v>
@@ -5929,7 +6024,7 @@
         <v>286</v>
       </c>
       <c r="T43" s="2" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="U43" s="10"/>
       <c r="V43" s="10"/>
@@ -5939,7 +6034,7 @@
     </row>
     <row r="44" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>319</v>
+        <v>338</v>
       </c>
       <c r="B44" s="10"/>
       <c r="C44" s="10"/>
@@ -5951,10 +6046,10 @@
       <c r="I44" s="10"/>
       <c r="J44" s="10"/>
       <c r="K44" s="2" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="M44" s="2" t="s">
         <v>94</v>
@@ -5963,7 +6058,7 @@
         <v>94</v>
       </c>
       <c r="O44" s="2" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="P44" s="2">
         <v>24.95</v>
@@ -5978,7 +6073,7 @@
         <v>399</v>
       </c>
       <c r="T44" s="2" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
       <c r="U44" s="10"/>
       <c r="V44" s="10"/>
@@ -5988,40 +6083,40 @@
     </row>
     <row r="45" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>334</v>
+        <v>353</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="H45" s="9" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="I45" s="9" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J45" s="9" t="s">
         <v>94</v>
       </c>
       <c r="K45" s="9" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L45" s="9" t="s">
-        <v>337</v>
+        <v>356</v>
       </c>
       <c r="M45" s="9" t="s">
         <v>94</v>
@@ -6030,7 +6125,7 @@
         <v>94</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>338</v>
+        <v>357</v>
       </c>
       <c r="P45" s="9">
         <v>49.95</v>
@@ -6045,7 +6140,7 @@
         <v>1438</v>
       </c>
       <c r="T45" s="9" t="s">
-        <v>339</v>
+        <v>358</v>
       </c>
       <c r="U45" s="9" t="s">
         <v>94</v>
@@ -6065,7 +6160,7 @@
     </row>
     <row r="46" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B46" s="10"/>
       <c r="C46" s="10"/>
@@ -6077,10 +6172,10 @@
       <c r="I46" s="10"/>
       <c r="J46" s="10"/>
       <c r="K46" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>340</v>
+        <v>359</v>
       </c>
       <c r="M46" s="2" t="s">
         <v>94</v>
@@ -6089,7 +6184,7 @@
         <v>94</v>
       </c>
       <c r="O46" s="2" t="s">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="P46" s="2">
         <v>49.95</v>
@@ -6104,7 +6199,7 @@
         <v>1438</v>
       </c>
       <c r="T46" s="2" t="s">
-        <v>342</v>
+        <v>361</v>
       </c>
       <c r="U46" s="10"/>
       <c r="V46" s="10"/>
@@ -6114,7 +6209,7 @@
     </row>
     <row r="47" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B47" s="10"/>
       <c r="C47" s="10"/>
@@ -6126,10 +6221,10 @@
       <c r="I47" s="10"/>
       <c r="J47" s="10"/>
       <c r="K47" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="M47" s="2" t="s">
         <v>94</v>
@@ -6138,7 +6233,7 @@
         <v>94</v>
       </c>
       <c r="O47" s="2" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="P47" s="2">
         <v>49.95</v>
@@ -6153,7 +6248,7 @@
         <v>1438</v>
       </c>
       <c r="T47" s="2" t="s">
-        <v>345</v>
+        <v>364</v>
       </c>
       <c r="U47" s="10"/>
       <c r="V47" s="10"/>
@@ -6163,7 +6258,7 @@
     </row>
     <row r="48" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B48" s="10"/>
       <c r="C48" s="10"/>
@@ -6175,10 +6270,10 @@
       <c r="I48" s="10"/>
       <c r="J48" s="10"/>
       <c r="K48" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>346</v>
+        <v>365</v>
       </c>
       <c r="M48" s="2" t="s">
         <v>94</v>
@@ -6187,7 +6282,7 @@
         <v>94</v>
       </c>
       <c r="O48" s="2" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="P48" s="2">
         <v>49.95</v>
@@ -6202,7 +6297,7 @@
         <v>1438</v>
       </c>
       <c r="T48" s="2" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="U48" s="10"/>
       <c r="V48" s="10"/>
@@ -6212,7 +6307,7 @@
     </row>
     <row r="49" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B49" s="10"/>
       <c r="C49" s="10"/>
@@ -6224,10 +6319,10 @@
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
       <c r="K49" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
       <c r="M49" s="2" t="s">
         <v>94</v>
@@ -6236,7 +6331,7 @@
         <v>94</v>
       </c>
       <c r="O49" s="2" t="s">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="P49" s="2">
         <v>49.95</v>
@@ -6251,7 +6346,7 @@
         <v>1438</v>
       </c>
       <c r="T49" s="2" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="U49" s="10"/>
       <c r="V49" s="10"/>
@@ -6261,7 +6356,7 @@
     </row>
     <row r="50" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B50" s="10"/>
       <c r="C50" s="10"/>
@@ -6273,10 +6368,10 @@
       <c r="I50" s="10"/>
       <c r="J50" s="10"/>
       <c r="K50" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>352</v>
+        <v>371</v>
       </c>
       <c r="M50" s="2" t="s">
         <v>94</v>
@@ -6285,7 +6380,7 @@
         <v>94</v>
       </c>
       <c r="O50" s="2" t="s">
-        <v>353</v>
+        <v>372</v>
       </c>
       <c r="P50" s="2">
         <v>49.95</v>
@@ -6300,7 +6395,7 @@
         <v>1438</v>
       </c>
       <c r="T50" s="2" t="s">
-        <v>354</v>
+        <v>373</v>
       </c>
       <c r="U50" s="10"/>
       <c r="V50" s="10"/>
@@ -6310,7 +6405,7 @@
     </row>
     <row r="51" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
@@ -6322,10 +6417,10 @@
       <c r="I51" s="10"/>
       <c r="J51" s="10"/>
       <c r="K51" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
       <c r="M51" s="2" t="s">
         <v>94</v>
@@ -6334,7 +6429,7 @@
         <v>94</v>
       </c>
       <c r="O51" s="2" t="s">
-        <v>356</v>
+        <v>375</v>
       </c>
       <c r="P51" s="2">
         <v>49.95</v>
@@ -6349,7 +6444,7 @@
         <v>1438</v>
       </c>
       <c r="T51" s="2" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
       <c r="U51" s="10"/>
       <c r="V51" s="10"/>
@@ -6359,7 +6454,7 @@
     </row>
     <row r="52" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
@@ -6371,10 +6466,10 @@
       <c r="I52" s="10"/>
       <c r="J52" s="10"/>
       <c r="K52" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>358</v>
+        <v>377</v>
       </c>
       <c r="M52" s="2" t="s">
         <v>94</v>
@@ -6383,7 +6478,7 @@
         <v>94</v>
       </c>
       <c r="O52" s="2" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
       <c r="P52" s="2">
         <v>49.95</v>
@@ -6398,7 +6493,7 @@
         <v>1438</v>
       </c>
       <c r="T52" s="2" t="s">
-        <v>360</v>
+        <v>379</v>
       </c>
       <c r="U52" s="10"/>
       <c r="V52" s="10"/>
@@ -6408,7 +6503,7 @@
     </row>
     <row r="53" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B53" s="10"/>
       <c r="C53" s="10"/>
@@ -6420,10 +6515,10 @@
       <c r="I53" s="10"/>
       <c r="J53" s="10"/>
       <c r="K53" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="M53" s="2" t="s">
         <v>94</v>
@@ -6432,7 +6527,7 @@
         <v>94</v>
       </c>
       <c r="O53" s="2" t="s">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="P53" s="2">
         <v>49.95</v>
@@ -6447,7 +6542,7 @@
         <v>1438</v>
       </c>
       <c r="T53" s="2" t="s">
-        <v>363</v>
+        <v>382</v>
       </c>
       <c r="U53" s="10"/>
       <c r="V53" s="10"/>
@@ -6457,7 +6552,7 @@
     </row>
     <row r="54" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B54" s="10"/>
       <c r="C54" s="10"/>
@@ -6469,10 +6564,10 @@
       <c r="I54" s="10"/>
       <c r="J54" s="10"/>
       <c r="K54" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>364</v>
+        <v>383</v>
       </c>
       <c r="M54" s="2" t="s">
         <v>94</v>
@@ -6481,7 +6576,7 @@
         <v>94</v>
       </c>
       <c r="O54" s="2" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="P54" s="2">
         <v>49.95</v>
@@ -6496,7 +6591,7 @@
         <v>1438</v>
       </c>
       <c r="T54" s="2" t="s">
-        <v>366</v>
+        <v>385</v>
       </c>
       <c r="U54" s="10"/>
       <c r="V54" s="10"/>
@@ -6506,7 +6601,7 @@
     </row>
     <row r="55" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B55" s="10"/>
       <c r="C55" s="10"/>
@@ -6518,10 +6613,10 @@
       <c r="I55" s="10"/>
       <c r="J55" s="10"/>
       <c r="K55" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>367</v>
+        <v>386</v>
       </c>
       <c r="M55" s="2" t="s">
         <v>94</v>
@@ -6530,7 +6625,7 @@
         <v>94</v>
       </c>
       <c r="O55" s="2" t="s">
-        <v>368</v>
+        <v>387</v>
       </c>
       <c r="P55" s="2">
         <v>49.95</v>
@@ -6545,7 +6640,7 @@
         <v>1438</v>
       </c>
       <c r="T55" s="2" t="s">
-        <v>369</v>
+        <v>388</v>
       </c>
       <c r="U55" s="10"/>
       <c r="V55" s="10"/>
@@ -6555,7 +6650,7 @@
     </row>
     <row r="56" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B56" s="10"/>
       <c r="C56" s="10"/>
@@ -6567,10 +6662,10 @@
       <c r="I56" s="10"/>
       <c r="J56" s="10"/>
       <c r="K56" s="2" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>370</v>
+        <v>389</v>
       </c>
       <c r="M56" s="2" t="s">
         <v>94</v>
@@ -6579,7 +6674,7 @@
         <v>94</v>
       </c>
       <c r="O56" s="2" t="s">
-        <v>371</v>
+        <v>390</v>
       </c>
       <c r="P56" s="2">
         <v>49.95</v>
@@ -6594,7 +6689,7 @@
         <v>1438</v>
       </c>
       <c r="T56" s="2" t="s">
-        <v>372</v>
+        <v>391</v>
       </c>
       <c r="U56" s="10"/>
       <c r="V56" s="10"/>
@@ -6602,250 +6697,6 @@
       <c r="X56" s="10"/>
       <c r="Y56" s="10"/>
     </row>
-    <row r="57" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="202" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="203" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="211" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="212" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="213" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="214" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="217" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="218" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="241" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="243" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="244" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="245" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="247" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="248" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="249" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="250" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="251" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="252" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="253" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="254" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="256" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="257" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="258" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="259" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="260" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="261" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="262" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="263" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="264" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="265" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="266" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="267" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="268" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="269" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="270" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="271" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="272" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="273" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="274" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="275" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="276" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="277" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="278" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="279" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="280" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="281" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="282" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="283" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="284" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="285" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="286" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="287" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="288" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="289" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="290" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="291" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="292" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="293" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="294" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="295" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="296" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="297" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="298" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="299" spans="3:9" x14ac:dyDescent="0.25"/>
-    <row r="300" spans="3:9" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <dataValidations count="8">
@@ -6875,7 +6726,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Admin UI: plain-language results with 'I know coding' switch, clearer preview text
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sienna-art-studio-admin/samples/sienna-products-import.xlsx
+++ b/sienna-art-studio-admin/samples/sienna-products-import.xlsx
@@ -503,7 +503,7 @@
     <t>Always run the Dry run first</t>
   </si>
   <si>
-    <t>Tick "Dry run" in the panel: it shows create / update for every row and writes nothing. Existing products must say update, only new ones create. If an old product says create, STOP and ask the developer.</t>
+    <t>Keep "Preview only (Dry run)" ticked in the panel and press "Run preview": it shows what would be added / updated and changes nothing. Then untick it and press "Import to the site". Old products must say "will be updated", only new ones "will be added". If an old product says "will be added", STOP and ask the developer.</t>
   </si>
   <si>
     <t>Product made in Shopify by hand</t>
@@ -515,7 +515,7 @@
     <t>Test with one product</t>
   </si>
   <si>
-    <t>In the panel, type the Product Code in "Only these product codes" to touch only that product. Leave it empty to import everything. Categories and the site menu are always updated.</t>
+    <t>In the panel, type the Product Code in "Only some products" to touch only that product. Leave it empty to import everything. Categories and the site menu are always updated.</t>
   </si>
   <si>
     <t>Name</t>

</xml_diff>